<commit_message>
F&O forward log: score the two tentative directional hints
The Summary now measures, per cycle and overall, the stock PCR gap (top
fifth minus bottom fifth, % up -- within one recording date) and the index
skew gap. Both stay out of the live view; the forward record decides.
October re-recorded the same day to include the volatility fields.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/history/fno_ranges.xlsx
+++ b/history/fno_ranges.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -435,6 +435,8 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,6 +485,16 @@
           <t>max_pain_closer_pct</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>tentative_hint</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>hint_gap_pts</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -502,7 +514,12 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>skew: top 40% minus rest, % up (backtest: about +17)</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -523,7 +540,12 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PCR: top fifth minus bottom fifth, % up (backtest: +5 to +6)</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -544,7 +566,12 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>skew: top 40% minus rest, % up (backtest: about +17)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -565,13 +592,18 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PCR: top fifth minus bottom fifth, % up (backtest: +5 to +6)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>One expiry is noise: stocks move together, so one large market move can push most of a cycle outside its range. Judge inside_range_pct against expected_hit_pct over several cycles. Walls held/max pain closer are positioning checks -- the backtest found no edge in them.</t>
+          <t>One expiry is noise: stocks move together, so one large market move can push most of a cycle outside its range. Judge inside_range_pct against expected_hit_pct over several cycles. Walls held/max pain closer are positioning checks -- the backtest found no edge in them. hint_gap_pts scores the two unconfirmed directional hints; they stay out of the live view until many cycles here agree with the backtest.</t>
         </is>
       </c>
     </row>
@@ -586,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:AD55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -595,7 +627,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -606,13 +638,19 @@
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="23" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="9" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="17" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -703,35 +741,65 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>iv_straddle_pct</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>iv_percentile</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>iv_rv</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>skew_pts</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>term_pts</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>results_before_expiry</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>expiry_close</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>ret_pct</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>inside_range</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>put_wall_held</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>call_wall_held</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>max_pain_closer</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>scored_on</t>
         </is>
@@ -742,13 +810,13 @@
         <v>46303</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46303.4499074074</v>
+        <v>46303.58364583334</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -761,22 +829,22 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>22457.7</v>
+        <v>22223.15</v>
       </c>
       <c r="H2" t="n">
-        <v>556.2</v>
+        <v>606.23</v>
       </c>
       <c r="I2" t="n">
-        <v>21901.5</v>
+        <v>21616.93</v>
       </c>
       <c r="J2" t="n">
-        <v>23013.9</v>
+        <v>22829.38</v>
       </c>
       <c r="K2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L2" t="n">
-        <v>13.4</v>
+        <v>14.7</v>
       </c>
       <c r="M2" t="n">
         <v>22000</v>
@@ -785,7 +853,7 @@
         <v>23500</v>
       </c>
       <c r="O2" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -795,19 +863,34 @@
       <c r="Q2" t="n">
         <v>23100</v>
       </c>
+      <c r="R2" t="n">
+        <v>15</v>
+      </c>
+      <c r="S2" t="n">
+        <v>76</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-0.6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46303.4499074074</v>
+        <v>46303.58417824074</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -820,22 +903,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>54893</v>
+        <v>54508.35</v>
       </c>
       <c r="H3" t="n">
-        <v>1536.75</v>
+        <v>1639.97</v>
       </c>
       <c r="I3" t="n">
-        <v>53356.25</v>
+        <v>52868.38</v>
       </c>
       <c r="J3" t="n">
-        <v>56429.75</v>
+        <v>56148.32</v>
       </c>
       <c r="K3" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L3" t="n">
-        <v>15.4</v>
+        <v>16.3</v>
       </c>
       <c r="M3" t="n">
         <v>52000</v>
@@ -844,7 +927,7 @@
         <v>58000</v>
       </c>
       <c r="O3" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -852,7 +935,22 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>55700</v>
+        <v>55500</v>
+      </c>
+      <c r="R3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="S3" t="n">
+        <v>73</v>
+      </c>
+      <c r="T3" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="V3" t="n">
+        <v>-0.8</v>
       </c>
     </row>
     <row r="4">
@@ -860,13 +958,13 @@
         <v>46303</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58364583334</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -879,53 +977,65 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>24793.3</v>
+        <v>24600.2</v>
       </c>
       <c r="H4" t="n">
-        <v>749.65</v>
+        <v>812.75</v>
       </c>
       <c r="I4" t="n">
-        <v>24043.65</v>
+        <v>23787.45</v>
       </c>
       <c r="J4" t="n">
-        <v>25542.95</v>
+        <v>25412.95</v>
       </c>
       <c r="K4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L4" t="n">
-        <v>16.7</v>
+        <v>18</v>
       </c>
       <c r="M4" t="n">
         <v>24600</v>
       </c>
       <c r="N4" t="n">
-        <v>25000</v>
+        <v>25100</v>
       </c>
       <c r="O4" t="n">
-        <v>1.28</v>
+        <v>1.09</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>bullish</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="Q4" t="n">
         <v>25000</v>
       </c>
+      <c r="R4" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>75</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58358796296</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -938,22 +1048,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>13605</v>
+        <v>13447.8</v>
       </c>
       <c r="H5" t="n">
-        <v>437.8</v>
+        <v>480.73</v>
       </c>
       <c r="I5" t="n">
-        <v>13167.2</v>
+        <v>12967.07</v>
       </c>
       <c r="J5" t="n">
-        <v>14042.8</v>
+        <v>13928.52</v>
       </c>
       <c r="K5" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L5" t="n">
-        <v>17.7</v>
+        <v>19.4</v>
       </c>
       <c r="M5" t="n">
         <v>12500</v>
@@ -962,7 +1072,7 @@
         <v>14500</v>
       </c>
       <c r="O5" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -972,19 +1082,31 @@
       <c r="Q5" t="n">
         <v>13900</v>
       </c>
+      <c r="R5" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="S5" t="n">
+        <v>77</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>46303.45010416667</v>
+        <v>46303.58405092593</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -997,31 +1119,31 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2634.9</v>
+        <v>2551.7</v>
       </c>
       <c r="H6" t="n">
-        <v>169.5</v>
+        <v>185.35</v>
       </c>
       <c r="I6" t="n">
-        <v>2465.4</v>
+        <v>2366.35</v>
       </c>
       <c r="J6" t="n">
-        <v>2804.4</v>
+        <v>2737.05</v>
       </c>
       <c r="K6" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L6" t="n">
-        <v>37.3</v>
+        <v>39.8</v>
       </c>
       <c r="M6" t="n">
-        <v>2600</v>
+        <v>2500</v>
       </c>
       <c r="N6" t="n">
         <v>2800</v>
       </c>
       <c r="O6" t="n">
-        <v>0.58</v>
+        <v>0.54</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1029,7 +1151,22 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>2800</v>
+        <v>2750</v>
+      </c>
+      <c r="R6" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="S6" t="n">
+        <v>87</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="U6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-3.3</v>
       </c>
     </row>
     <row r="7">
@@ -1037,13 +1174,13 @@
         <v>46303</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>46303.45013888889</v>
+        <v>46303.58405092593</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1056,31 +1193,31 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1708.3</v>
+        <v>1682.5</v>
       </c>
       <c r="H7" t="n">
-        <v>80.75</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>1627.55</v>
+        <v>1597.9</v>
       </c>
       <c r="J7" t="n">
-        <v>1789.05</v>
+        <v>1767.1</v>
       </c>
       <c r="K7" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L7" t="n">
-        <v>26.2</v>
+        <v>27.6</v>
       </c>
       <c r="M7" t="n">
-        <v>1700</v>
+        <v>1680</v>
       </c>
       <c r="N7" t="n">
         <v>1800</v>
       </c>
       <c r="O7" t="n">
-        <v>0.78</v>
+        <v>0.73</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1090,19 +1227,34 @@
       <c r="Q7" t="n">
         <v>1760</v>
       </c>
+      <c r="R7" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="S7" t="n">
+        <v>74</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="U7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>46303.45028935185</v>
+        <v>46303.58393518518</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1115,31 +1267,31 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>7802.5</v>
+        <v>7631</v>
       </c>
       <c r="H8" t="n">
-        <v>327.5</v>
+        <v>344.5</v>
       </c>
       <c r="I8" t="n">
-        <v>7475</v>
+        <v>7286.5</v>
       </c>
       <c r="J8" t="n">
-        <v>8130</v>
+        <v>7975.5</v>
       </c>
       <c r="K8" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L8" t="n">
-        <v>22.7</v>
+        <v>24.5</v>
       </c>
       <c r="M8" t="n">
-        <v>7800</v>
+        <v>7000</v>
       </c>
       <c r="N8" t="n">
-        <v>8500</v>
+        <v>8000</v>
       </c>
       <c r="O8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1147,7 +1299,22 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>8100</v>
+        <v>8000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="S8" t="n">
+        <v>80</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-1.8</v>
       </c>
     </row>
     <row r="9">
@@ -1155,13 +1322,13 @@
         <v>46303</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>46303.45032407407</v>
+        <v>46303.58358796296</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1174,22 +1341,22 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2355.9</v>
+        <v>2323.8</v>
       </c>
       <c r="H9" t="n">
-        <v>92.83</v>
+        <v>96.83</v>
       </c>
       <c r="I9" t="n">
-        <v>2263.08</v>
+        <v>2226.98</v>
       </c>
       <c r="J9" t="n">
-        <v>2448.72</v>
+        <v>2420.62</v>
       </c>
       <c r="K9" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L9" t="n">
-        <v>21.8</v>
+        <v>22.9</v>
       </c>
       <c r="M9" t="n">
         <v>2300</v>
@@ -1198,29 +1365,44 @@
         <v>2400</v>
       </c>
       <c r="O9" t="n">
-        <v>0.52</v>
+        <v>0.49</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>bearish</t>
         </is>
       </c>
       <c r="Q9" t="n">
         <v>2400</v>
       </c>
+      <c r="R9" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="S9" t="n">
+        <v>60</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58375</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1233,31 +1415,31 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1247.4</v>
+        <v>1240.7</v>
       </c>
       <c r="H10" t="n">
-        <v>57.12</v>
+        <v>58.38</v>
       </c>
       <c r="I10" t="n">
-        <v>1190.28</v>
+        <v>1182.33</v>
       </c>
       <c r="J10" t="n">
-        <v>1304.53</v>
+        <v>1299.08</v>
       </c>
       <c r="K10" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L10" t="n">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="M10" t="n">
-        <v>1220</v>
+        <v>1200</v>
       </c>
       <c r="N10" t="n">
         <v>1260</v>
       </c>
       <c r="O10" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1267,19 +1449,39 @@
       <c r="Q10" t="n">
         <v>1220</v>
       </c>
+      <c r="R10" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="S10" t="n">
+        <v>81</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="U10" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>17-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58384259259</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1292,31 +1494,31 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>9819</v>
+        <v>9695</v>
       </c>
       <c r="H11" t="n">
-        <v>381.15</v>
+        <v>401.17</v>
       </c>
       <c r="I11" t="n">
-        <v>9437.85</v>
+        <v>9293.83</v>
       </c>
       <c r="J11" t="n">
-        <v>10200.15</v>
+        <v>10096.17</v>
       </c>
       <c r="K11" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L11" t="n">
-        <v>21.1</v>
+        <v>22.6</v>
       </c>
       <c r="M11" t="n">
-        <v>9800</v>
+        <v>9000</v>
       </c>
       <c r="N11" t="n">
         <v>10500</v>
       </c>
       <c r="O11" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1324,7 +1526,27 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>10200</v>
+        <v>10100</v>
+      </c>
+      <c r="R11" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="S11" t="n">
+        <v>56</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-0</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>27-Oct</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1332,13 +1554,13 @@
         <v>46303</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>46303.45032407407</v>
+        <v>46303.58388888889</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1351,22 +1573,22 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1717.4</v>
+        <v>1703.7</v>
       </c>
       <c r="H12" t="n">
-        <v>75.17</v>
+        <v>77.73</v>
       </c>
       <c r="I12" t="n">
-        <v>1642.23</v>
+        <v>1625.98</v>
       </c>
       <c r="J12" t="n">
-        <v>1792.58</v>
+        <v>1781.42</v>
       </c>
       <c r="K12" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L12" t="n">
-        <v>24.3</v>
+        <v>24.9</v>
       </c>
       <c r="M12" t="n">
         <v>1700</v>
@@ -1375,7 +1597,7 @@
         <v>1840</v>
       </c>
       <c r="O12" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1385,19 +1607,34 @@
       <c r="Q12" t="n">
         <v>1780</v>
       </c>
+      <c r="R12" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>80</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="U12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>46303.45055555556</v>
+        <v>46303.58364583334</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1410,22 +1647,22 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>958.1</v>
+        <v>951.2</v>
       </c>
       <c r="H13" t="n">
-        <v>52.6</v>
+        <v>53.9</v>
       </c>
       <c r="I13" t="n">
-        <v>905.5</v>
+        <v>897.3</v>
       </c>
       <c r="J13" t="n">
-        <v>1010.7</v>
+        <v>1005.1</v>
       </c>
       <c r="K13" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L13" t="n">
-        <v>30</v>
+        <v>31.2</v>
       </c>
       <c r="M13" t="n">
         <v>940</v>
@@ -1434,7 +1671,7 @@
         <v>1000</v>
       </c>
       <c r="O13" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1444,19 +1681,39 @@
       <c r="Q13" t="n">
         <v>980</v>
       </c>
+      <c r="R13" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>83</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V13" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>19-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1469,31 +1726,31 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>374.05</v>
+        <v>367.95</v>
       </c>
       <c r="H14" t="n">
-        <v>17.75</v>
+        <v>18.1</v>
       </c>
       <c r="I14" t="n">
-        <v>356.3</v>
+        <v>349.85</v>
       </c>
       <c r="J14" t="n">
-        <v>391.8</v>
+        <v>386.05</v>
       </c>
       <c r="K14" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L14" t="n">
-        <v>26.1</v>
+        <v>27</v>
       </c>
       <c r="M14" t="n">
-        <v>370</v>
+        <v>340</v>
       </c>
       <c r="N14" t="n">
         <v>400</v>
       </c>
       <c r="O14" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -1503,19 +1760,34 @@
       <c r="Q14" t="n">
         <v>390</v>
       </c>
+      <c r="R14" t="n">
+        <v>27</v>
+      </c>
+      <c r="S14" t="n">
+        <v>62</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="V14" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>46303.45055555556</v>
+        <v>46303.58405092593</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1528,31 +1800,31 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1820.2</v>
+        <v>1799.7</v>
       </c>
       <c r="H15" t="n">
-        <v>49.62</v>
+        <v>49.8</v>
       </c>
       <c r="I15" t="n">
-        <v>1770.58</v>
+        <v>1749.9</v>
       </c>
       <c r="J15" t="n">
-        <v>1869.83</v>
+        <v>1849.5</v>
       </c>
       <c r="K15" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L15" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="M15" t="n">
-        <v>1820</v>
+        <v>1780</v>
       </c>
       <c r="N15" t="n">
         <v>1840</v>
       </c>
       <c r="O15" t="n">
-        <v>0.67</v>
+        <v>0.64</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -1562,19 +1834,34 @@
       <c r="Q15" t="n">
         <v>1820</v>
       </c>
+      <c r="R15" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="S15" t="n">
+        <v>19</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="U15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V15" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58364583334</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1587,31 +1874,31 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>3370.7</v>
+        <v>3317.4</v>
       </c>
       <c r="H16" t="n">
-        <v>228.68</v>
+        <v>223.1</v>
       </c>
       <c r="I16" t="n">
-        <v>3142.02</v>
+        <v>3094.3</v>
       </c>
       <c r="J16" t="n">
-        <v>3599.38</v>
+        <v>3540.5</v>
       </c>
       <c r="K16" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L16" t="n">
-        <v>37.1</v>
+        <v>36.7</v>
       </c>
       <c r="M16" t="n">
-        <v>3200</v>
+        <v>3000</v>
       </c>
       <c r="N16" t="n">
         <v>3500</v>
       </c>
       <c r="O16" t="n">
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -1621,19 +1908,34 @@
       <c r="Q16" t="n">
         <v>3200</v>
       </c>
+      <c r="R16" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="S16" t="n">
+        <v>46</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="U16" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>46303.45045138889</v>
+        <v>46303.58451388889</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1646,22 +1948,22 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1317.9</v>
+        <v>1294.5</v>
       </c>
       <c r="H17" t="n">
-        <v>56.98</v>
+        <v>59.38</v>
       </c>
       <c r="I17" t="n">
-        <v>1260.93</v>
+        <v>1235.12</v>
       </c>
       <c r="J17" t="n">
-        <v>1374.88</v>
+        <v>1353.88</v>
       </c>
       <c r="K17" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L17" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="M17" t="n">
         <v>1220</v>
@@ -1670,7 +1972,7 @@
         <v>1400</v>
       </c>
       <c r="O17" t="n">
-        <v>0.66</v>
+        <v>0.64</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -1680,19 +1982,39 @@
       <c r="Q17" t="n">
         <v>1350</v>
       </c>
+      <c r="R17" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="S17" t="n">
+        <v>81</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>27-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>46303.45025462963</v>
+        <v>46303.58417824074</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1705,22 +2027,22 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>407.05</v>
+        <v>407.3</v>
       </c>
       <c r="H18" t="n">
-        <v>16.62</v>
+        <v>17.25</v>
       </c>
       <c r="I18" t="n">
-        <v>390.43</v>
+        <v>390.05</v>
       </c>
       <c r="J18" t="n">
-        <v>423.68</v>
+        <v>424.55</v>
       </c>
       <c r="K18" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L18" t="n">
-        <v>21.8</v>
+        <v>22.9</v>
       </c>
       <c r="M18" t="n">
         <v>400</v>
@@ -1729,7 +2051,7 @@
         <v>430</v>
       </c>
       <c r="O18" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -1739,19 +2061,34 @@
       <c r="Q18" t="n">
         <v>420</v>
       </c>
+      <c r="R18" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="S18" t="n">
+        <v>65</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-1.7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>46303.45037037037</v>
+        <v>46303.58364583334</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1764,22 +2101,22 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1190.2</v>
+        <v>1176.7</v>
       </c>
       <c r="H19" t="n">
-        <v>57.95</v>
+        <v>58.3</v>
       </c>
       <c r="I19" t="n">
-        <v>1132.25</v>
+        <v>1118.4</v>
       </c>
       <c r="J19" t="n">
-        <v>1248.15</v>
+        <v>1235</v>
       </c>
       <c r="K19" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L19" t="n">
-        <v>27.2</v>
+        <v>27.3</v>
       </c>
       <c r="M19" t="n">
         <v>1100</v>
@@ -1788,7 +2125,7 @@
         <v>1200</v>
       </c>
       <c r="O19" t="n">
-        <v>0.67</v>
+        <v>0.7</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -1798,19 +2135,39 @@
       <c r="Q19" t="n">
         <v>1200</v>
       </c>
+      <c r="R19" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="S19" t="n">
+        <v>83</v>
+      </c>
+      <c r="T19" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>23-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>46303.4509375</v>
+        <v>46303.58405092593</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1823,22 +2180,22 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>6923</v>
+        <v>6853.5</v>
       </c>
       <c r="H20" t="n">
-        <v>269.1</v>
+        <v>277.68</v>
       </c>
       <c r="I20" t="n">
-        <v>6653.9</v>
+        <v>6575.82</v>
       </c>
       <c r="J20" t="n">
-        <v>7192.1</v>
+        <v>7131.18</v>
       </c>
       <c r="K20" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L20" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="M20" t="n">
         <v>6600</v>
@@ -1847,7 +2204,7 @@
         <v>7500</v>
       </c>
       <c r="O20" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -1857,19 +2214,34 @@
       <c r="Q20" t="n">
         <v>7200</v>
       </c>
+      <c r="R20" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="S20" t="n">
+        <v>46</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V20" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>46303.45032407407</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C21" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D21" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1882,31 +2254,31 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>325.3</v>
+        <v>321.3</v>
       </c>
       <c r="H21" t="n">
-        <v>19.48</v>
+        <v>20.28</v>
       </c>
       <c r="I21" t="n">
-        <v>305.82</v>
+        <v>301.03</v>
       </c>
       <c r="J21" t="n">
-        <v>344.78</v>
+        <v>341.57</v>
       </c>
       <c r="K21" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L21" t="n">
-        <v>32.8</v>
+        <v>34.6</v>
       </c>
       <c r="M21" t="n">
         <v>320</v>
       </c>
       <c r="N21" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="O21" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
@@ -1916,19 +2288,34 @@
       <c r="Q21" t="n">
         <v>325</v>
       </c>
+      <c r="R21" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="S21" t="n">
+        <v>63</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="U21" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-1.5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>46303.45101851852</v>
+        <v>46303.58400462963</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1941,22 +2328,22 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2887</v>
+        <v>2875.5</v>
       </c>
       <c r="H22" t="n">
-        <v>112.2</v>
+        <v>110.5</v>
       </c>
       <c r="I22" t="n">
-        <v>2774.8</v>
+        <v>2765</v>
       </c>
       <c r="J22" t="n">
-        <v>2999.2</v>
+        <v>2986</v>
       </c>
       <c r="K22" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L22" t="n">
-        <v>22.8</v>
+        <v>20.9</v>
       </c>
       <c r="M22" t="n">
         <v>2800</v>
@@ -1965,7 +2352,7 @@
         <v>3000</v>
       </c>
       <c r="O22" t="n">
-        <v>0.6</v>
+        <v>0.54</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -1975,19 +2362,34 @@
       <c r="Q22" t="n">
         <v>3000</v>
       </c>
+      <c r="R22" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>58</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="U22" t="n">
+        <v>2</v>
+      </c>
+      <c r="V22" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>46303.45101851852</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2000,22 +2402,22 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1204.9</v>
+        <v>1189.5</v>
       </c>
       <c r="H23" t="n">
-        <v>79.45</v>
+        <v>80.05</v>
       </c>
       <c r="I23" t="n">
-        <v>1125.45</v>
+        <v>1109.45</v>
       </c>
       <c r="J23" t="n">
-        <v>1284.35</v>
+        <v>1269.55</v>
       </c>
       <c r="K23" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L23" t="n">
-        <v>36.1</v>
+        <v>36.8</v>
       </c>
       <c r="M23" t="n">
         <v>1100</v>
@@ -2024,7 +2426,7 @@
         <v>1250</v>
       </c>
       <c r="O23" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -2034,19 +2436,39 @@
       <c r="Q23" t="n">
         <v>1220</v>
       </c>
+      <c r="R23" t="n">
+        <v>37</v>
+      </c>
+      <c r="S23" t="n">
+        <v>97</v>
+      </c>
+      <c r="T23" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="U23" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="V23" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>12-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>46303.45055555556</v>
+        <v>46303.58462962963</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2059,22 +2481,22 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>695.9</v>
+        <v>691.1</v>
       </c>
       <c r="H24" t="n">
-        <v>30.35</v>
+        <v>30.38</v>
       </c>
       <c r="I24" t="n">
-        <v>665.55</v>
+        <v>660.73</v>
       </c>
       <c r="J24" t="n">
-        <v>726.25</v>
+        <v>721.48</v>
       </c>
       <c r="K24" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L24" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="M24" t="n">
         <v>670</v>
@@ -2093,19 +2515,39 @@
       <c r="Q24" t="n">
         <v>720</v>
       </c>
+      <c r="R24" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="S24" t="n">
+        <v>77</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="U24" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="V24" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>17-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>46303.45101851852</v>
+        <v>46303.58399305555</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D25" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2118,22 +2560,22 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>546.25</v>
+        <v>545.35</v>
       </c>
       <c r="H25" t="n">
-        <v>27.98</v>
+        <v>29.5</v>
       </c>
       <c r="I25" t="n">
-        <v>518.27</v>
+        <v>515.85</v>
       </c>
       <c r="J25" t="n">
-        <v>574.23</v>
+        <v>574.85</v>
       </c>
       <c r="K25" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L25" t="n">
-        <v>28.1</v>
+        <v>29.7</v>
       </c>
       <c r="M25" t="n">
         <v>500</v>
@@ -2142,7 +2584,7 @@
         <v>560</v>
       </c>
       <c r="O25" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -2152,19 +2594,39 @@
       <c r="Q25" t="n">
         <v>535</v>
       </c>
+      <c r="R25" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="S25" t="n">
+        <v>94</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="U25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V25" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>15-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>46303.45086805556</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C26" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D26" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2177,22 +2639,22 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>901.75</v>
+        <v>890.8</v>
       </c>
       <c r="H26" t="n">
-        <v>45.35</v>
+        <v>46.02</v>
       </c>
       <c r="I26" t="n">
-        <v>856.4</v>
+        <v>844.77</v>
       </c>
       <c r="J26" t="n">
-        <v>947.1</v>
+        <v>936.8200000000001</v>
       </c>
       <c r="K26" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L26" t="n">
-        <v>27.5</v>
+        <v>28.2</v>
       </c>
       <c r="M26" t="n">
         <v>850</v>
@@ -2201,7 +2663,7 @@
         <v>960</v>
       </c>
       <c r="O26" t="n">
-        <v>0.98</v>
+        <v>0.89</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
@@ -2211,19 +2673,34 @@
       <c r="Q26" t="n">
         <v>960</v>
       </c>
+      <c r="R26" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="S26" t="n">
+        <v>60</v>
+      </c>
+      <c r="T26" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="U26" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>46303.45086805556</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D27" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2236,25 +2713,25 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1863.3</v>
+        <v>1846.4</v>
       </c>
       <c r="H27" t="n">
-        <v>63.05</v>
+        <v>64</v>
       </c>
       <c r="I27" t="n">
-        <v>1800.25</v>
+        <v>1782.4</v>
       </c>
       <c r="J27" t="n">
-        <v>1926.35</v>
+        <v>1910.4</v>
       </c>
       <c r="K27" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L27" t="n">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
       <c r="M27" t="n">
-        <v>1860</v>
+        <v>1840</v>
       </c>
       <c r="N27" t="n">
         <v>2000</v>
@@ -2270,19 +2747,34 @@
       <c r="Q27" t="n">
         <v>1900</v>
       </c>
+      <c r="R27" t="n">
+        <v>19</v>
+      </c>
+      <c r="S27" t="n">
+        <v>50</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="U27" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="V27" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>46303.45086805556</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D28" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2295,22 +2787,22 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1354.8</v>
+        <v>1343.3</v>
       </c>
       <c r="H28" t="n">
-        <v>52.8</v>
+        <v>53.75</v>
       </c>
       <c r="I28" t="n">
-        <v>1302</v>
+        <v>1289.55</v>
       </c>
       <c r="J28" t="n">
-        <v>1407.6</v>
+        <v>1397.05</v>
       </c>
       <c r="K28" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L28" t="n">
-        <v>21</v>
+        <v>21.8</v>
       </c>
       <c r="M28" t="n">
         <v>1300</v>
@@ -2319,7 +2811,7 @@
         <v>1400</v>
       </c>
       <c r="O28" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
@@ -2329,19 +2821,39 @@
       <c r="Q28" t="n">
         <v>1340</v>
       </c>
+      <c r="R28" t="n">
+        <v>22</v>
+      </c>
+      <c r="S28" t="n">
+        <v>81</v>
+      </c>
+      <c r="T28" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="U28" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V28" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>17-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B29" s="3" t="n">
-        <v>46303.45090277777</v>
+        <v>46303.58462962963</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D29" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2354,31 +2866,31 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>4901.7</v>
+        <v>4815.4</v>
       </c>
       <c r="H29" t="n">
-        <v>245.33</v>
+        <v>261.25</v>
       </c>
       <c r="I29" t="n">
-        <v>4656.38</v>
+        <v>4554.15</v>
       </c>
       <c r="J29" t="n">
-        <v>5147.02</v>
+        <v>5076.65</v>
       </c>
       <c r="K29" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L29" t="n">
-        <v>27.8</v>
+        <v>29.5</v>
       </c>
       <c r="M29" t="n">
-        <v>4900</v>
+        <v>4800</v>
       </c>
       <c r="N29" t="n">
         <v>5100</v>
       </c>
       <c r="O29" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
@@ -2388,19 +2900,34 @@
       <c r="Q29" t="n">
         <v>5000</v>
       </c>
+      <c r="R29" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="S29" t="n">
+        <v>71</v>
+      </c>
+      <c r="T29" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="U29" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="V29" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>46303.45090277777</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C30" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D30" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2413,53 +2940,73 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1006.75</v>
+        <v>999.75</v>
       </c>
       <c r="H30" t="n">
-        <v>68.25</v>
+        <v>68.22</v>
       </c>
       <c r="I30" t="n">
-        <v>938.5</v>
+        <v>931.52</v>
       </c>
       <c r="J30" t="n">
-        <v>1075</v>
+        <v>1067.97</v>
       </c>
       <c r="K30" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L30" t="n">
-        <v>37.1</v>
+        <v>37.5</v>
       </c>
       <c r="M30" t="n">
-        <v>1000</v>
+        <v>960</v>
       </c>
       <c r="N30" t="n">
         <v>1040</v>
       </c>
       <c r="O30" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>bullish</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="Q30" t="n">
         <v>1020</v>
       </c>
+      <c r="R30" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="S30" t="n">
+        <v>92</v>
+      </c>
+      <c r="T30" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="U30" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="V30" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>23-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>46303.45079861111</v>
+        <v>46303.58400462963</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D31" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2472,22 +3019,22 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>257.2</v>
+        <v>254.05</v>
       </c>
       <c r="H31" t="n">
-        <v>9.800000000000001</v>
+        <v>10.15</v>
       </c>
       <c r="I31" t="n">
-        <v>247.4</v>
+        <v>243.9</v>
       </c>
       <c r="J31" t="n">
-        <v>267</v>
+        <v>264.2</v>
       </c>
       <c r="K31" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L31" t="n">
-        <v>20.7</v>
+        <v>21.8</v>
       </c>
       <c r="M31" t="n">
         <v>250</v>
@@ -2496,7 +3043,7 @@
         <v>270</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
@@ -2504,7 +3051,22 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>265</v>
+        <v>262.5</v>
+      </c>
+      <c r="R31" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="S31" t="n">
+        <v>88</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="U31" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="V31" t="n">
+        <v>-0.5</v>
       </c>
     </row>
     <row r="32">
@@ -2512,13 +3074,13 @@
         <v>46303</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>46303.4509375</v>
+        <v>46303.58451388889</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2531,22 +3093,22 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>213.81</v>
+        <v>211.06</v>
       </c>
       <c r="H32" t="n">
-        <v>11.88</v>
+        <v>12.29</v>
       </c>
       <c r="I32" t="n">
-        <v>201.94</v>
+        <v>198.78</v>
       </c>
       <c r="J32" t="n">
-        <v>225.69</v>
+        <v>223.34</v>
       </c>
       <c r="K32" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L32" t="n">
-        <v>30.7</v>
+        <v>31.5</v>
       </c>
       <c r="M32" t="n">
         <v>210</v>
@@ -2565,19 +3127,34 @@
       <c r="Q32" t="n">
         <v>225</v>
       </c>
+      <c r="R32" t="n">
+        <v>32</v>
+      </c>
+      <c r="S32" t="n">
+        <v>75</v>
+      </c>
+      <c r="T32" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="U32" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="V32" t="n">
+        <v>-1.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>46303.45113425926</v>
+        <v>46303.58439814814</v>
       </c>
       <c r="C33" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D33" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2590,22 +3167,22 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>1203.1</v>
+        <v>1178.3</v>
       </c>
       <c r="H33" t="n">
-        <v>58.52</v>
+        <v>60.27</v>
       </c>
       <c r="I33" t="n">
-        <v>1144.57</v>
+        <v>1118.02</v>
       </c>
       <c r="J33" t="n">
-        <v>1261.62</v>
+        <v>1238.58</v>
       </c>
       <c r="K33" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L33" t="n">
-        <v>27.4</v>
+        <v>28.1</v>
       </c>
       <c r="M33" t="n">
         <v>1120</v>
@@ -2614,15 +3191,35 @@
         <v>1280</v>
       </c>
       <c r="O33" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>1240</v>
+      </c>
+      <c r="R33" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="S33" t="n">
+        <v>78</v>
+      </c>
+      <c r="T33" t="n">
         <v>0.97</v>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>bullish</t>
-        </is>
-      </c>
-      <c r="Q33" t="n">
-        <v>1260</v>
+      <c r="U33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>-3</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>23-Oct</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -2630,13 +3227,13 @@
         <v>46303</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>46303.45101851852</v>
+        <v>46303.58423611111</v>
       </c>
       <c r="C34" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2649,22 +3246,22 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>436.5</v>
+        <v>434.6</v>
       </c>
       <c r="H34" t="n">
-        <v>17.95</v>
+        <v>18.32</v>
       </c>
       <c r="I34" t="n">
-        <v>418.55</v>
+        <v>416.28</v>
       </c>
       <c r="J34" t="n">
-        <v>454.45</v>
+        <v>452.93</v>
       </c>
       <c r="K34" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L34" t="n">
-        <v>22.5</v>
+        <v>23</v>
       </c>
       <c r="M34" t="n">
         <v>430</v>
@@ -2673,7 +3270,7 @@
         <v>440</v>
       </c>
       <c r="O34" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
@@ -2683,19 +3280,34 @@
       <c r="Q34" t="n">
         <v>420</v>
       </c>
+      <c r="R34" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="S34" t="n">
+        <v>66</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="U34" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="V34" t="n">
+        <v>-0.6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>46303.45125</v>
+        <v>46303.58497685185</v>
       </c>
       <c r="C35" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D35" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2708,31 +3320,31 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>3666.7</v>
+        <v>3631.3</v>
       </c>
       <c r="H35" t="n">
-        <v>148.7</v>
+        <v>148.5</v>
       </c>
       <c r="I35" t="n">
-        <v>3518</v>
+        <v>3482.8</v>
       </c>
       <c r="J35" t="n">
-        <v>3815.4</v>
+        <v>3779.8</v>
       </c>
       <c r="K35" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L35" t="n">
-        <v>22.1</v>
+        <v>22.4</v>
       </c>
       <c r="M35" t="n">
         <v>3400</v>
       </c>
       <c r="N35" t="n">
-        <v>4000</v>
+        <v>3800</v>
       </c>
       <c r="O35" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
@@ -2742,19 +3354,34 @@
       <c r="Q35" t="n">
         <v>3850</v>
       </c>
+      <c r="R35" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="S35" t="n">
+        <v>74</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="U35" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>46303.45125</v>
+        <v>46303.58501157408</v>
       </c>
       <c r="C36" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D36" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2767,22 +3394,22 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>2788.1</v>
+        <v>2753.5</v>
       </c>
       <c r="H36" t="n">
-        <v>119.95</v>
+        <v>123.02</v>
       </c>
       <c r="I36" t="n">
-        <v>2668.15</v>
+        <v>2630.47</v>
       </c>
       <c r="J36" t="n">
-        <v>2908.05</v>
+        <v>2876.53</v>
       </c>
       <c r="K36" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L36" t="n">
-        <v>23.5</v>
+        <v>24.3</v>
       </c>
       <c r="M36" t="n">
         <v>2700</v>
@@ -2791,7 +3418,7 @@
         <v>3000</v>
       </c>
       <c r="O36" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
@@ -2801,19 +3428,34 @@
       <c r="Q36" t="n">
         <v>2900</v>
       </c>
+      <c r="R36" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="S36" t="n">
+        <v>58</v>
+      </c>
+      <c r="T36" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="U36" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="V36" t="n">
+        <v>2.3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>46303.45125</v>
+        <v>46303.58524305555</v>
       </c>
       <c r="C37" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D37" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2826,22 +3468,22 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>11339</v>
+        <v>11250</v>
       </c>
       <c r="H37" t="n">
-        <v>479.3</v>
+        <v>491.35</v>
       </c>
       <c r="I37" t="n">
-        <v>10859.7</v>
+        <v>10758.65</v>
       </c>
       <c r="J37" t="n">
-        <v>11818.3</v>
+        <v>11741.35</v>
       </c>
       <c r="K37" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L37" t="n">
-        <v>23</v>
+        <v>23.7</v>
       </c>
       <c r="M37" t="n">
         <v>11000</v>
@@ -2850,15 +3492,30 @@
         <v>12000</v>
       </c>
       <c r="O37" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>bearish</t>
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>11800</v>
+        <v>11700</v>
+      </c>
+      <c r="R37" t="n">
+        <v>24</v>
+      </c>
+      <c r="S37" t="n">
+        <v>75</v>
+      </c>
+      <c r="T37" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="U37" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="V37" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="38">
@@ -2866,13 +3523,13 @@
         <v>46303</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>46303.4509375</v>
+        <v>46303.5850462963</v>
       </c>
       <c r="C38" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D38" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2885,22 +3542,22 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>888.75</v>
+        <v>874.35</v>
       </c>
       <c r="H38" t="n">
-        <v>52.18</v>
+        <v>53.05</v>
       </c>
       <c r="I38" t="n">
-        <v>836.58</v>
+        <v>821.3</v>
       </c>
       <c r="J38" t="n">
-        <v>940.92</v>
+        <v>927.4</v>
       </c>
       <c r="K38" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L38" t="n">
-        <v>32.3</v>
+        <v>33.1</v>
       </c>
       <c r="M38" t="n">
         <v>800</v>
@@ -2909,7 +3566,7 @@
         <v>900</v>
       </c>
       <c r="O38" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
@@ -2919,19 +3576,34 @@
       <c r="Q38" t="n">
         <v>930</v>
       </c>
+      <c r="R38" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="S38" t="n">
+        <v>92</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="U38" t="n">
+        <v>1</v>
+      </c>
+      <c r="V38" t="n">
+        <v>-2.1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>46303.45112268518</v>
+        <v>46303.58532407408</v>
       </c>
       <c r="C39" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D39" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2944,22 +3616,22 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1335.9</v>
+        <v>1315.6</v>
       </c>
       <c r="H39" t="n">
-        <v>64.72</v>
+        <v>65.78</v>
       </c>
       <c r="I39" t="n">
-        <v>1271.18</v>
+        <v>1249.82</v>
       </c>
       <c r="J39" t="n">
-        <v>1400.62</v>
+        <v>1381.38</v>
       </c>
       <c r="K39" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L39" t="n">
-        <v>26.6</v>
+        <v>27.4</v>
       </c>
       <c r="M39" t="n">
         <v>1300</v>
@@ -2968,7 +3640,7 @@
         <v>1400</v>
       </c>
       <c r="O39" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
@@ -2978,19 +3650,39 @@
       <c r="Q39" t="n">
         <v>1330</v>
       </c>
+      <c r="R39" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="S39" t="n">
+        <v>91</v>
+      </c>
+      <c r="T39" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V39" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>15-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58532407408</v>
       </c>
       <c r="C40" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -3003,31 +3695,31 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>313.6</v>
+        <v>312.2</v>
       </c>
       <c r="H40" t="n">
-        <v>11.28</v>
+        <v>11.65</v>
       </c>
       <c r="I40" t="n">
-        <v>302.33</v>
+        <v>300.55</v>
       </c>
       <c r="J40" t="n">
-        <v>324.88</v>
+        <v>323.85</v>
       </c>
       <c r="K40" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L40" t="n">
-        <v>19.3</v>
+        <v>20.4</v>
       </c>
       <c r="M40" t="n">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="N40" t="n">
         <v>325</v>
       </c>
       <c r="O40" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
@@ -3037,19 +3729,34 @@
       <c r="Q40" t="n">
         <v>325</v>
       </c>
+      <c r="R40" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="S40" t="n">
+        <v>70</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="U40" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="V40" t="n">
+        <v>9.699999999999999</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58532407408</v>
       </c>
       <c r="C41" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D41" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -3062,31 +3769,31 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>220.71</v>
+        <v>219.25</v>
       </c>
       <c r="H41" t="n">
-        <v>8.359999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>212.36</v>
+        <v>210.47</v>
       </c>
       <c r="J41" t="n">
-        <v>229.06</v>
+        <v>228.03</v>
       </c>
       <c r="K41" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L41" t="n">
-        <v>20.7</v>
+        <v>22.1</v>
       </c>
       <c r="M41" t="n">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="N41" t="n">
         <v>240</v>
       </c>
       <c r="O41" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
@@ -3096,19 +3803,34 @@
       <c r="Q41" t="n">
         <v>227.5</v>
       </c>
+      <c r="R41" t="n">
+        <v>22</v>
+      </c>
+      <c r="S41" t="n">
+        <v>55</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V41" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58532407408</v>
       </c>
       <c r="C42" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D42" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -3121,31 +3843,31 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>247.8</v>
+        <v>246.35</v>
       </c>
       <c r="H42" t="n">
-        <v>9.970000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="I42" t="n">
-        <v>237.83</v>
+        <v>236.15</v>
       </c>
       <c r="J42" t="n">
-        <v>257.78</v>
+        <v>256.55</v>
       </c>
       <c r="K42" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L42" t="n">
-        <v>21.8</v>
+        <v>22.9</v>
       </c>
       <c r="M42" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="N42" t="n">
         <v>270</v>
       </c>
       <c r="O42" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
@@ -3155,19 +3877,34 @@
       <c r="Q42" t="n">
         <v>260</v>
       </c>
+      <c r="R42" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="S42" t="n">
+        <v>76</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1</v>
+      </c>
+      <c r="V42" t="n">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>46303.45109953704</v>
+        <v>46303.58532407408</v>
       </c>
       <c r="C43" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D43" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -3180,22 +3917,22 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>1189.2</v>
+        <v>1175.8</v>
       </c>
       <c r="H43" t="n">
-        <v>48.8</v>
+        <v>49.67</v>
       </c>
       <c r="I43" t="n">
-        <v>1140.4</v>
+        <v>1126.12</v>
       </c>
       <c r="J43" t="n">
-        <v>1238</v>
+        <v>1225.47</v>
       </c>
       <c r="K43" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L43" t="n">
-        <v>22.4</v>
+        <v>23</v>
       </c>
       <c r="M43" t="n">
         <v>1160</v>
@@ -3204,7 +3941,7 @@
         <v>1250</v>
       </c>
       <c r="O43" t="n">
-        <v>0.76</v>
+        <v>0.73</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
@@ -3212,7 +3949,22 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>1230</v>
+        <v>1220</v>
+      </c>
+      <c r="R43" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="S43" t="n">
+        <v>76</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1</v>
+      </c>
+      <c r="U43" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="V43" t="n">
+        <v>-1.1</v>
       </c>
     </row>
     <row r="44">
@@ -3220,13 +3972,13 @@
         <v>46303</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58520833333</v>
       </c>
       <c r="C44" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3239,31 +3991,31 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1673.7</v>
+        <v>1670.3</v>
       </c>
       <c r="H44" t="n">
-        <v>82.62</v>
+        <v>84.48</v>
       </c>
       <c r="I44" t="n">
-        <v>1591.08</v>
+        <v>1585.83</v>
       </c>
       <c r="J44" t="n">
-        <v>1756.33</v>
+        <v>1754.77</v>
       </c>
       <c r="K44" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L44" t="n">
-        <v>27.3</v>
+        <v>27.2</v>
       </c>
       <c r="M44" t="n">
-        <v>1600</v>
+        <v>1640</v>
       </c>
       <c r="N44" t="n">
         <v>1800</v>
       </c>
       <c r="O44" t="n">
-        <v>0.62</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P44" t="inlineStr">
         <is>
@@ -3273,19 +4025,34 @@
       <c r="Q44" t="n">
         <v>1740</v>
       </c>
+      <c r="R44" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="S44" t="n">
+        <v>92</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="U44" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="V44" t="n">
+        <v>-3.2</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>46303.45090277777</v>
+        <v>46303.58578703704</v>
       </c>
       <c r="C45" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -3298,22 +4065,22 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>950</v>
+        <v>941.1</v>
       </c>
       <c r="H45" t="n">
-        <v>35.72</v>
+        <v>36.98</v>
       </c>
       <c r="I45" t="n">
-        <v>914.27</v>
+        <v>904.12</v>
       </c>
       <c r="J45" t="n">
-        <v>985.73</v>
+        <v>978.08</v>
       </c>
       <c r="K45" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L45" t="n">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="M45" t="n">
         <v>940</v>
@@ -3322,29 +4089,44 @@
         <v>1000</v>
       </c>
       <c r="O45" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>bullish</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="Q45" t="n">
         <v>980</v>
       </c>
+      <c r="R45" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="S45" t="n">
+        <v>55</v>
+      </c>
+      <c r="T45" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="U45" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="V45" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>46303.45140046296</v>
+        <v>46303.58543981481</v>
       </c>
       <c r="C46" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D46" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3357,22 +4139,22 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>933.8</v>
+        <v>920.05</v>
       </c>
       <c r="H46" t="n">
-        <v>52.92</v>
+        <v>54.15</v>
       </c>
       <c r="I46" t="n">
-        <v>880.88</v>
+        <v>865.9</v>
       </c>
       <c r="J46" t="n">
-        <v>986.72</v>
+        <v>974.2</v>
       </c>
       <c r="K46" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L46" t="n">
-        <v>31.2</v>
+        <v>32.2</v>
       </c>
       <c r="M46" t="n">
         <v>920</v>
@@ -3381,7 +4163,7 @@
         <v>1000</v>
       </c>
       <c r="O46" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="P46" t="inlineStr">
         <is>
@@ -3391,19 +4173,34 @@
       <c r="Q46" t="n">
         <v>980</v>
       </c>
+      <c r="R46" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="S46" t="n">
+        <v>67</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="U46" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V46" t="n">
+        <v>-0.5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>46303.45097222222</v>
+        <v>46303.58578703704</v>
       </c>
       <c r="C47" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D47" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -3416,22 +4213,22 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>1779</v>
+        <v>1751.2</v>
       </c>
       <c r="H47" t="n">
-        <v>58.3</v>
+        <v>59.9</v>
       </c>
       <c r="I47" t="n">
-        <v>1720.7</v>
+        <v>1691.3</v>
       </c>
       <c r="J47" t="n">
-        <v>1837.3</v>
+        <v>1811.1</v>
       </c>
       <c r="K47" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L47" t="n">
-        <v>17.9</v>
+        <v>18.7</v>
       </c>
       <c r="M47" t="n">
         <v>1660</v>
@@ -3440,7 +4237,7 @@
         <v>1900</v>
       </c>
       <c r="O47" t="n">
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
       <c r="P47" t="inlineStr">
         <is>
@@ -3448,7 +4245,22 @@
         </is>
       </c>
       <c r="Q47" t="n">
-        <v>1820</v>
+        <v>1800</v>
+      </c>
+      <c r="R47" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="S47" t="n">
+        <v>73</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="U47" t="n">
+        <v>1</v>
+      </c>
+      <c r="V47" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="48">
@@ -3456,13 +4268,13 @@
         <v>46303</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>46303.45101851852</v>
+        <v>46303.58543981481</v>
       </c>
       <c r="C48" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D48" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3475,28 +4287,28 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>966.65</v>
+        <v>949.05</v>
       </c>
       <c r="H48" t="n">
-        <v>38.97</v>
+        <v>40.8</v>
       </c>
       <c r="I48" t="n">
-        <v>927.67</v>
+        <v>908.25</v>
       </c>
       <c r="J48" t="n">
-        <v>1005.62</v>
+        <v>989.85</v>
       </c>
       <c r="K48" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L48" t="n">
-        <v>22</v>
+        <v>23.2</v>
       </c>
       <c r="M48" t="n">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="N48" t="n">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="O48" t="n">
         <v>0.75</v>
@@ -3509,19 +4321,34 @@
       <c r="Q48" t="n">
         <v>990</v>
       </c>
+      <c r="R48" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="S48" t="n">
+        <v>65</v>
+      </c>
+      <c r="T48" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="U48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V48" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B49" s="3" t="n">
-        <v>46303.45106481481</v>
+        <v>46303.58543981481</v>
       </c>
       <c r="C49" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D49" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -3534,31 +4361,31 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>174.91</v>
+        <v>172.46</v>
       </c>
       <c r="H49" t="n">
-        <v>8.949999999999999</v>
+        <v>9.41</v>
       </c>
       <c r="I49" t="n">
-        <v>165.96</v>
+        <v>163.05</v>
       </c>
       <c r="J49" t="n">
-        <v>183.86</v>
+        <v>181.87</v>
       </c>
       <c r="K49" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L49" t="n">
-        <v>28.3</v>
+        <v>29.9</v>
       </c>
       <c r="M49" t="n">
         <v>170</v>
       </c>
       <c r="N49" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="O49" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="P49" t="inlineStr">
         <is>
@@ -3568,19 +4395,34 @@
       <c r="Q49" t="n">
         <v>182.5</v>
       </c>
+      <c r="R49" t="n">
+        <v>30</v>
+      </c>
+      <c r="S49" t="n">
+        <v>81</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="U49" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V49" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B50" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58543981481</v>
       </c>
       <c r="C50" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -3593,22 +4435,22 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2115.5</v>
+        <v>2103</v>
       </c>
       <c r="H50" t="n">
-        <v>122.2</v>
+        <v>124</v>
       </c>
       <c r="I50" t="n">
-        <v>1993.3</v>
+        <v>1979</v>
       </c>
       <c r="J50" t="n">
-        <v>2237.7</v>
+        <v>2227</v>
       </c>
       <c r="K50" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L50" t="n">
-        <v>31.8</v>
+        <v>32.1</v>
       </c>
       <c r="M50" t="n">
         <v>2100</v>
@@ -3617,7 +4459,7 @@
         <v>2200</v>
       </c>
       <c r="O50" t="n">
-        <v>0.72</v>
+        <v>0.66</v>
       </c>
       <c r="P50" t="inlineStr">
         <is>
@@ -3627,19 +4469,39 @@
       <c r="Q50" t="n">
         <v>2100</v>
       </c>
+      <c r="R50" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="S50" t="n">
+        <v>91</v>
+      </c>
+      <c r="T50" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="U50" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="V50" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>08-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B51" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58556712963</v>
       </c>
       <c r="C51" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D51" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -3652,22 +4514,22 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1516.8</v>
+        <v>1503.7</v>
       </c>
       <c r="H51" t="n">
-        <v>92</v>
+        <v>94.8</v>
       </c>
       <c r="I51" t="n">
-        <v>1424.8</v>
+        <v>1408.9</v>
       </c>
       <c r="J51" t="n">
-        <v>1608.8</v>
+        <v>1598.5</v>
       </c>
       <c r="K51" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L51" t="n">
-        <v>33.7</v>
+        <v>34.5</v>
       </c>
       <c r="M51" t="n">
         <v>1500</v>
@@ -3676,7 +4538,7 @@
         <v>1540</v>
       </c>
       <c r="O51" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="P51" t="inlineStr">
         <is>
@@ -3686,19 +4548,39 @@
       <c r="Q51" t="n">
         <v>1520</v>
       </c>
+      <c r="R51" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="S51" t="n">
+        <v>92</v>
+      </c>
+      <c r="T51" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="U51" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="V51" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>15-Oct</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>46303.45113425926</v>
+        <v>46303.58608796296</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D52" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -3711,22 +4593,22 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>4429.2</v>
+        <v>4379.2</v>
       </c>
       <c r="H52" t="n">
-        <v>155.07</v>
+        <v>165.05</v>
       </c>
       <c r="I52" t="n">
-        <v>4274.12</v>
+        <v>4214.15</v>
       </c>
       <c r="J52" t="n">
-        <v>4584.27</v>
+        <v>4544.25</v>
       </c>
       <c r="K52" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L52" t="n">
-        <v>19</v>
+        <v>20.6</v>
       </c>
       <c r="M52" t="n">
         <v>4300</v>
@@ -3735,7 +4617,7 @@
         <v>4500</v>
       </c>
       <c r="O52" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="P52" t="inlineStr">
         <is>
@@ -3745,19 +4627,34 @@
       <c r="Q52" t="n">
         <v>4500</v>
       </c>
+      <c r="R52" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="S52" t="n">
+        <v>51</v>
+      </c>
+      <c r="T52" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="U52" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="V52" t="n">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B53" s="3" t="n">
-        <v>46303.45136574074</v>
+        <v>46303.58596064815</v>
       </c>
       <c r="C53" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D53" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -3770,31 +4667,31 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>280.55</v>
+        <v>274.8</v>
       </c>
       <c r="H53" t="n">
-        <v>14.8</v>
+        <v>15.25</v>
       </c>
       <c r="I53" t="n">
-        <v>265.75</v>
+        <v>259.55</v>
       </c>
       <c r="J53" t="n">
-        <v>295.35</v>
+        <v>290.05</v>
       </c>
       <c r="K53" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L53" t="n">
-        <v>29</v>
+        <v>30.5</v>
       </c>
       <c r="M53" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="N53" t="n">
         <v>300</v>
       </c>
       <c r="O53" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="P53" t="inlineStr">
         <is>
@@ -3804,19 +4701,34 @@
       <c r="Q53" t="n">
         <v>290</v>
       </c>
+      <c r="R53" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="S53" t="n">
+        <v>59</v>
+      </c>
+      <c r="T53" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="U53" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="V53" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>46303.45100694444</v>
+        <v>46303.58578703704</v>
       </c>
       <c r="C54" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D54" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -3829,31 +4741,31 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>2930.8</v>
+        <v>2890.1</v>
       </c>
       <c r="H54" t="n">
-        <v>139.28</v>
+        <v>138.68</v>
       </c>
       <c r="I54" t="n">
-        <v>2791.53</v>
+        <v>2751.42</v>
       </c>
       <c r="J54" t="n">
-        <v>3070.08</v>
+        <v>3028.78</v>
       </c>
       <c r="K54" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L54" t="n">
-        <v>26.1</v>
+        <v>26.8</v>
       </c>
       <c r="M54" t="n">
         <v>2800</v>
       </c>
       <c r="N54" t="n">
-        <v>3000</v>
+        <v>2900</v>
       </c>
       <c r="O54" t="n">
-        <v>0.93</v>
+        <v>0.88</v>
       </c>
       <c r="P54" t="inlineStr">
         <is>
@@ -3863,19 +4775,34 @@
       <c r="Q54" t="n">
         <v>2850</v>
       </c>
+      <c r="R54" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="S54" t="n">
+        <v>31</v>
+      </c>
+      <c r="T54" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="U54" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="V54" t="n">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="B55" s="3" t="n">
-        <v>46303.45148148148</v>
+        <v>46303.58556712963</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>46322</v>
       </c>
       <c r="D55" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -3888,22 +4815,22 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>10580</v>
+        <v>10538</v>
       </c>
       <c r="H55" t="n">
-        <v>464.55</v>
+        <v>475.5</v>
       </c>
       <c r="I55" t="n">
-        <v>10115.45</v>
+        <v>10062.5</v>
       </c>
       <c r="J55" t="n">
-        <v>11044.55</v>
+        <v>11013.5</v>
       </c>
       <c r="K55" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L55" t="n">
-        <v>24.1</v>
+        <v>24.4</v>
       </c>
       <c r="M55" t="n">
         <v>9800</v>
@@ -3912,7 +4839,7 @@
         <v>11500</v>
       </c>
       <c r="O55" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -3921,6 +4848,26 @@
       </c>
       <c r="Q55" t="n">
         <v>11000</v>
+      </c>
+      <c r="R55" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="S55" t="n">
+        <v>76</v>
+      </c>
+      <c r="T55" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="U55" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="V55" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>19-Oct</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>